<commit_message>
Update market dashboard data
</commit_message>
<xml_diff>
--- a/output/exports/setup_summary.xlsx
+++ b/output/exports/setup_summary.xlsx
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>499</v>
+        <v>487</v>
       </c>
     </row>
     <row r="6">
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>